<commit_message>
更新看板 10月11日 — KPI272.9万(17.9%) 净流水243.8万
</commit_message>
<xml_diff>
--- a/导出_总表.xlsx
+++ b/导出_总表.xlsx
@@ -525,7 +525,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1400000</v>
+        <v>1450000</v>
       </c>
       <c r="D2" t="n">
         <v>242888</v>
@@ -541,12 +541,12 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>17.3%</t>
+          <t>16.8%</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>17.3%</t>
+          <t>16.8%</t>
         </is>
       </c>
       <c r="J2" t="n">
@@ -979,7 +979,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>800000</v>
+        <v>1030000</v>
       </c>
       <c r="D10" t="n">
         <v>51229</v>
@@ -993,12 +993,12 @@
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
-          <t>-2.8%</t>
+          <t>-2.2%</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>-2.8%</t>
+          <t>-2.2%</t>
         </is>
       </c>
       <c r="J10" t="n">
@@ -1156,7 +1156,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>700000</v>
+        <v>1600000</v>
       </c>
       <c r="D13" t="n">
         <v>87201</v>
@@ -1170,12 +1170,12 @@
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr">
         <is>
-          <t>10.9%</t>
+          <t>4.8%</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>10.9%</t>
+          <t>4.8%</t>
         </is>
       </c>
       <c r="J13" t="n">
@@ -1447,7 +1447,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>14090000</v>
+        <v>15270000</v>
       </c>
       <c r="D18" t="n">
         <v>2964140</v>
@@ -1463,12 +1463,12 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>17.3%</t>
+          <t>16.0%</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>17.3%</t>
+          <t>16.0%</t>
         </is>
       </c>
       <c r="J18" t="n">
@@ -2097,7 +2097,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>191500</v>
+        <v>312912</v>
       </c>
       <c r="D2" t="n">
         <v>74994</v>
@@ -2107,12 +2107,12 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>39.2%</t>
+          <t>24.0%</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>39.2%</t>
+          <t>24.0%</t>
         </is>
       </c>
       <c r="H2" t="n">
@@ -2139,7 +2139,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>185200</v>
+        <v>302618</v>
       </c>
       <c r="D3" t="n">
         <v>6260</v>
@@ -2149,12 +2149,12 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>3.4%</t>
+          <t>2.1%</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>3.4%</t>
+          <t>2.1%</t>
         </is>
       </c>
       <c r="H3" t="n">
@@ -2181,7 +2181,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>165200</v>
+        <v>269938</v>
       </c>
       <c r="D4" t="n">
         <v>34860</v>
@@ -2191,12 +2191,12 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>21.1%</t>
+          <t>12.9%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>21.1%</t>
+          <t>12.9%</t>
         </is>
       </c>
       <c r="H4" t="n">
@@ -2223,7 +2223,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>98625</v>
+        <v>161154</v>
       </c>
       <c r="D5" t="n">
         <v>22000</v>
@@ -2233,12 +2233,12 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>22.3%</t>
+          <t>13.7%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>22.3%</t>
+          <t>13.7%</t>
         </is>
       </c>
       <c r="H5" t="n">
@@ -2265,7 +2265,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>98625</v>
+        <v>161154</v>
       </c>
       <c r="D6" t="n">
         <v>14940</v>
@@ -2275,12 +2275,12 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>15.1%</t>
+          <t>9.3%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>15.1%</t>
+          <t>9.3%</t>
         </is>
       </c>
       <c r="H6" t="n">
@@ -2307,7 +2307,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>148350</v>
+        <v>242405</v>
       </c>
       <c r="D7" t="n">
         <v>4681</v>
@@ -2317,12 +2317,12 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>3.2%</t>
+          <t>1.9%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>3.2%</t>
+          <t>1.9%</t>
         </is>
       </c>
       <c r="H7" t="n">
@@ -2349,7 +2349,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>115750</v>
+        <v>189136</v>
       </c>
       <c r="D8" t="n">
         <v>4980</v>
@@ -2359,12 +2359,12 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>4.3%</t>
+          <t>2.6%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>4.3%</t>
+          <t>2.6%</t>
         </is>
       </c>
       <c r="H8" t="n">
@@ -2391,7 +2391,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>207250</v>
+        <v>333616</v>
       </c>
       <c r="D9" t="n">
         <v>32976</v>
@@ -2401,12 +2401,12 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>15.9%</t>
+          <t>9.9%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>15.9%</t>
+          <t>9.9%</t>
         </is>
       </c>
       <c r="H9" t="n">
@@ -2433,7 +2433,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>168625</v>
+        <v>271440</v>
       </c>
       <c r="D10" t="n">
         <v>4980</v>
@@ -2443,12 +2443,12 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>3.0%</t>
+          <t>1.8%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>3.0%</t>
+          <t>1.8%</t>
         </is>
       </c>
       <c r="H10" t="n">
@@ -2475,7 +2475,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>168625</v>
+        <v>271440</v>
       </c>
       <c r="D11" t="n">
         <v>4980</v>
@@ -2485,12 +2485,12 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>3.0%</t>
+          <t>1.8%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>3.0%</t>
+          <t>1.8%</t>
         </is>
       </c>
       <c r="H11" t="n">
@@ -2517,7 +2517,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>148625</v>
+        <v>239246</v>
       </c>
       <c r="D12" t="n">
         <v>9960</v>
@@ -2527,12 +2527,12 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>6.7%</t>
+          <t>4.2%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>6.7%</t>
+          <t>4.2%</t>
         </is>
       </c>
       <c r="H12" t="n">
@@ -2559,7 +2559,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>141500</v>
+        <v>227777</v>
       </c>
       <c r="D13" t="n">
         <v>0</v>
@@ -2601,7 +2601,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>128625</v>
+        <v>207051</v>
       </c>
       <c r="D14" t="n">
         <v>9960</v>
@@ -2611,12 +2611,12 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>7.7%</t>
+          <t>4.8%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>7.7%</t>
+          <t>4.8%</t>
         </is>
       </c>
       <c r="H14" t="n">
@@ -2643,7 +2643,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>91500</v>
+        <v>147291</v>
       </c>
       <c r="D15" t="n">
         <v>6600</v>
@@ -2653,12 +2653,12 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>7.2%</t>
+          <t>4.5%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>7.2%</t>
+          <t>4.5%</t>
         </is>
       </c>
       <c r="H15" t="n">
@@ -2685,7 +2685,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>171500</v>
+        <v>279050</v>
       </c>
       <c r="D16" t="n">
         <v>24940</v>
@@ -2695,12 +2695,12 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>14.5%</t>
+          <t>8.9%</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>14.5%</t>
+          <t>8.9%</t>
         </is>
       </c>
       <c r="H16" t="n">
@@ -2727,7 +2727,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>175475</v>
+        <v>285517</v>
       </c>
       <c r="D17" t="n">
         <v>84074</v>
@@ -2737,12 +2737,12 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>47.9%</t>
+          <t>29.4%</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>47.9%</t>
+          <t>29.4%</t>
         </is>
       </c>
       <c r="H17" t="n">
@@ -2769,7 +2769,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>178625</v>
+        <v>290643</v>
       </c>
       <c r="D18" t="n">
         <v>25696</v>
@@ -2779,12 +2779,12 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>14.4%</t>
+          <t>8.8%</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>14.4%</t>
+          <t>8.8%</t>
         </is>
       </c>
       <c r="H18" t="n">
@@ -2811,7 +2811,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>178900</v>
+        <v>291091</v>
       </c>
       <c r="D19" t="n">
         <v>4980</v>
@@ -2821,12 +2821,12 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2.8%</t>
+          <t>1.7%</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2.8%</t>
+          <t>1.7%</t>
         </is>
       </c>
       <c r="H19" t="n">
@@ -2853,7 +2853,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>108625</v>
+        <v>176745</v>
       </c>
       <c r="D20" t="n">
         <v>14940</v>
@@ -2863,12 +2863,12 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>13.8%</t>
+          <t>8.5%</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>13.8%</t>
+          <t>8.5%</t>
         </is>
       </c>
       <c r="H20" t="n">
@@ -2895,7 +2895,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>95750</v>
+        <v>155796</v>
       </c>
       <c r="D21" t="n">
         <v>9960</v>
@@ -2905,12 +2905,12 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>10.4%</t>
+          <t>6.4%</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>10.4%</t>
+          <t>6.4%</t>
         </is>
       </c>
       <c r="H21" t="n">
@@ -2937,7 +2937,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>98625</v>
+        <v>160474</v>
       </c>
       <c r="D22" t="n">
         <v>14940</v>
@@ -2947,12 +2947,12 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>15.1%</t>
+          <t>9.3%</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>15.1%</t>
+          <t>9.3%</t>
         </is>
       </c>
       <c r="H22" t="n">
@@ -2979,7 +2979,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>207895</v>
+        <v>265322</v>
       </c>
       <c r="D23" t="n">
         <v>36178</v>
@@ -2989,12 +2989,12 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>17.4%</t>
+          <t>13.6%</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>17.4%</t>
+          <t>13.6%</t>
         </is>
       </c>
       <c r="H23" t="n">
@@ -3021,7 +3021,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>104842</v>
+        <v>133802</v>
       </c>
       <c r="D24" t="n">
         <v>33420</v>
@@ -3031,12 +3031,12 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>31.9%</t>
+          <t>25.0%</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>31.9%</t>
+          <t>25.0%</t>
         </is>
       </c>
       <c r="H24" t="n">
@@ -3063,7 +3063,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>100737</v>
+        <v>128563</v>
       </c>
       <c r="D25" t="n">
         <v>38000</v>
@@ -3073,12 +3073,12 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>37.7%</t>
+          <t>29.6%</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>37.7%</t>
+          <t>29.6%</t>
         </is>
       </c>
       <c r="H25" t="n">
@@ -3105,7 +3105,7 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>154842</v>
+        <v>197614</v>
       </c>
       <c r="D26" t="n">
         <v>24000</v>
@@ -3115,12 +3115,12 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>15.5%</t>
+          <t>12.1%</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>15.5%</t>
+          <t>12.1%</t>
         </is>
       </c>
       <c r="H26" t="n">
@@ -3147,7 +3147,7 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>150737</v>
+        <v>192375</v>
       </c>
       <c r="D27" t="n">
         <v>66400</v>
@@ -3157,12 +3157,12 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>44.1%</t>
+          <t>34.5%</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>44.1%</t>
+          <t>34.5%</t>
         </is>
       </c>
       <c r="H27" t="n">
@@ -3189,7 +3189,7 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>80000</v>
+        <v>102098</v>
       </c>
       <c r="D28" t="n">
         <v>0</v>
@@ -3231,7 +3231,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>80000</v>
+        <v>102098</v>
       </c>
       <c r="D29" t="n">
         <v>12000</v>
@@ -3241,12 +3241,12 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>15.0%</t>
+          <t>11.8%</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>15.0%</t>
+          <t>11.8%</t>
         </is>
       </c>
       <c r="H29" t="n">
@@ -3273,7 +3273,7 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>108947</v>
+        <v>139041</v>
       </c>
       <c r="D30" t="n">
         <v>6600</v>
@@ -3283,12 +3283,12 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>6.1%</t>
+          <t>4.7%</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>6.1%</t>
+          <t>4.7%</t>
         </is>
       </c>
       <c r="H30" t="n">
@@ -3315,7 +3315,7 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>80000</v>
+        <v>102098</v>
       </c>
       <c r="D31" t="n">
         <v>24088</v>
@@ -3325,12 +3325,12 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>30.1%</t>
+          <t>23.6%</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>30.1%</t>
+          <t>23.6%</t>
         </is>
       </c>
       <c r="H31" t="n">
@@ -3357,7 +3357,7 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>80000</v>
+        <v>102098</v>
       </c>
       <c r="D32" t="n">
         <v>43800</v>
@@ -3367,12 +3367,12 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>54.8%</t>
+          <t>42.9%</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>54.8%</t>
+          <t>42.9%</t>
         </is>
       </c>
       <c r="H32" t="n">
@@ -3399,7 +3399,7 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>80000</v>
+        <v>102098</v>
       </c>
       <c r="D33" t="n">
         <v>24800</v>
@@ -3409,12 +3409,12 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>31.0%</t>
+          <t>24.3%</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>31.0%</t>
+          <t>24.3%</t>
         </is>
       </c>
       <c r="H33" t="n">
@@ -3441,7 +3441,7 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>80000</v>
+        <v>102098</v>
       </c>
       <c r="D34" t="n">
         <v>0</v>
@@ -3483,7 +3483,7 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>80000</v>
+        <v>102098</v>
       </c>
       <c r="D35" t="n">
         <v>0</v>
@@ -3525,7 +3525,7 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>80000</v>
+        <v>102103</v>
       </c>
       <c r="D36" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
更新看板 10月11日 — KPI296.4万(17.2%) 净流水243.8万
</commit_message>
<xml_diff>
--- a/导出_总表.xlsx
+++ b/导出_总表.xlsx
@@ -737,7 +737,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>2000000</v>
+        <v>2500000</v>
       </c>
       <c r="D6" t="n">
         <v>590420</v>
@@ -751,12 +751,12 @@
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
-          <t>29.5%</t>
+          <t>23.6%</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>29.5%</t>
+          <t>23.6%</t>
         </is>
       </c>
       <c r="J6" t="n">
@@ -798,7 +798,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>380000</v>
+        <v>500000</v>
       </c>
       <c r="D7" t="n">
         <v>57135</v>
@@ -812,12 +812,12 @@
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
-          <t>14.1%</t>
+          <t>11.4%</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>14.1%</t>
+          <t>11.4%</t>
         </is>
       </c>
       <c r="J7" t="n">
@@ -859,7 +859,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>400000</v>
+        <v>600000</v>
       </c>
       <c r="D8" t="n">
         <v>236801</v>
@@ -873,12 +873,12 @@
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
-          <t>59.2%</t>
+          <t>39.5%</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>59.2%</t>
+          <t>39.5%</t>
         </is>
       </c>
       <c r="J8" t="n">
@@ -916,7 +916,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>800000</v>
+        <v>1000000</v>
       </c>
       <c r="D9" t="n">
         <v>193702</v>
@@ -930,12 +930,12 @@
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
-          <t>20.1%</t>
+          <t>19.4%</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>20.1%</t>
+          <t>19.4%</t>
         </is>
       </c>
       <c r="J9" t="n">
@@ -979,7 +979,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>1030000</v>
+        <v>1100000</v>
       </c>
       <c r="D10" t="n">
         <v>51229</v>
@@ -993,12 +993,12 @@
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
-          <t>-2.2%</t>
+          <t>4.7%</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>-2.2%</t>
+          <t>4.7%</t>
         </is>
       </c>
       <c r="J10" t="n">
@@ -1042,7 +1042,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>260000</v>
+        <v>400000</v>
       </c>
       <c r="D11" t="n">
         <v>16952</v>
@@ -1056,12 +1056,12 @@
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
         <is>
-          <t>3.8%</t>
+          <t>4.2%</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>3.8%</t>
+          <t>4.2%</t>
         </is>
       </c>
       <c r="J11" t="n">
@@ -1099,7 +1099,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>400000</v>
+        <v>500000</v>
       </c>
       <c r="D12" t="n">
         <v>150397</v>
@@ -1113,12 +1113,12 @@
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr">
         <is>
-          <t>35.3%</t>
+          <t>30.1%</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>35.3%</t>
+          <t>30.1%</t>
         </is>
       </c>
       <c r="J12" t="n">
@@ -1156,7 +1156,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1600000</v>
+        <v>1900000</v>
       </c>
       <c r="D13" t="n">
         <v>87201</v>
@@ -1170,12 +1170,12 @@
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr">
         <is>
-          <t>4.8%</t>
+          <t>4.6%</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>4.8%</t>
+          <t>4.6%</t>
         </is>
       </c>
       <c r="J13" t="n">
@@ -1219,7 +1219,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>900000</v>
+        <v>1000000</v>
       </c>
       <c r="D14" t="n">
         <v>478418</v>
@@ -1233,12 +1233,12 @@
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr">
         <is>
-          <t>46.4%</t>
+          <t>47.8%</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>46.4%</t>
+          <t>47.8%</t>
         </is>
       </c>
       <c r="J14" t="n">
@@ -1292,12 +1292,12 @@
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr">
         <is>
-          <t>15.1%</t>
+          <t>18.5%</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>15.1%</t>
+          <t>18.5%</t>
         </is>
       </c>
       <c r="J15" t="n">
@@ -1341,7 +1341,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>700000</v>
+        <v>900000</v>
       </c>
       <c r="D16" t="n">
         <v>41715</v>
@@ -1355,12 +1355,12 @@
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr">
         <is>
-          <t>6.0%</t>
+          <t>4.6%</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>6.0%</t>
+          <t>4.6%</t>
         </is>
       </c>
       <c r="J16" t="n">
@@ -1447,7 +1447,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>15270000</v>
+        <v>17200000</v>
       </c>
       <c r="D18" t="n">
         <v>2964140</v>
@@ -1463,12 +1463,12 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>16.0%</t>
+          <t>14.2%</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>16.0%</t>
+          <t>14.2%</t>
         </is>
       </c>
       <c r="J18" t="n">
@@ -2097,7 +2097,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>312912</v>
+        <v>3129120000</v>
       </c>
       <c r="D2" t="n">
         <v>74994</v>
@@ -2107,12 +2107,12 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>24.0%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>24.0%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="H2" t="n">
@@ -2139,7 +2139,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>302618</v>
+        <v>3026180000</v>
       </c>
       <c r="D3" t="n">
         <v>6260</v>
@@ -2149,12 +2149,12 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2.1%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2.1%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="H3" t="n">
@@ -2181,7 +2181,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>269938</v>
+        <v>2699380000</v>
       </c>
       <c r="D4" t="n">
         <v>34860</v>
@@ -2191,12 +2191,12 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>12.9%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>12.9%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="H4" t="n">
@@ -2223,7 +2223,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>161154</v>
+        <v>1611540000</v>
       </c>
       <c r="D5" t="n">
         <v>22000</v>
@@ -2233,12 +2233,12 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>13.7%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>13.7%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="H5" t="n">
@@ -2265,7 +2265,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>161154</v>
+        <v>1611540000</v>
       </c>
       <c r="D6" t="n">
         <v>14940</v>
@@ -2275,12 +2275,12 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>9.3%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>9.3%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="H6" t="n">
@@ -2307,7 +2307,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>242405</v>
+        <v>2424050000</v>
       </c>
       <c r="D7" t="n">
         <v>4681</v>
@@ -2317,12 +2317,12 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>1.9%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>1.9%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="H7" t="n">
@@ -2349,7 +2349,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>189136</v>
+        <v>1891360000</v>
       </c>
       <c r="D8" t="n">
         <v>4980</v>
@@ -2359,12 +2359,12 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2.6%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2.6%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="H8" t="n">
@@ -2391,7 +2391,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>333616</v>
+        <v>3336160000</v>
       </c>
       <c r="D9" t="n">
         <v>32976</v>
@@ -2401,12 +2401,12 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>9.9%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>9.9%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="H9" t="n">
@@ -2433,7 +2433,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>271440</v>
+        <v>2714400000</v>
       </c>
       <c r="D10" t="n">
         <v>4980</v>
@@ -2443,12 +2443,12 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>1.8%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>1.8%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="H10" t="n">
@@ -2475,7 +2475,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>271440</v>
+        <v>2714400000</v>
       </c>
       <c r="D11" t="n">
         <v>4980</v>
@@ -2485,12 +2485,12 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>1.8%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>1.8%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="H11" t="n">
@@ -2517,7 +2517,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>239246</v>
+        <v>2392460000</v>
       </c>
       <c r="D12" t="n">
         <v>9960</v>
@@ -2527,12 +2527,12 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>4.2%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>4.2%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="H12" t="n">
@@ -2559,7 +2559,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>227777</v>
+        <v>2277770000</v>
       </c>
       <c r="D13" t="n">
         <v>0</v>
@@ -2601,7 +2601,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>207051</v>
+        <v>2070510000</v>
       </c>
       <c r="D14" t="n">
         <v>9960</v>
@@ -2611,12 +2611,12 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>4.8%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>4.8%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="H14" t="n">
@@ -2643,7 +2643,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>147291</v>
+        <v>1472910000</v>
       </c>
       <c r="D15" t="n">
         <v>6600</v>
@@ -2653,12 +2653,12 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>4.5%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>4.5%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="H15" t="n">
@@ -2685,7 +2685,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>279050</v>
+        <v>2790500000</v>
       </c>
       <c r="D16" t="n">
         <v>24940</v>
@@ -2695,12 +2695,12 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>8.9%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>8.9%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="H16" t="n">
@@ -2727,7 +2727,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>285517</v>
+        <v>2855170000</v>
       </c>
       <c r="D17" t="n">
         <v>84074</v>
@@ -2737,12 +2737,12 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>29.4%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>29.4%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="H17" t="n">
@@ -2769,7 +2769,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>290643</v>
+        <v>2906430000</v>
       </c>
       <c r="D18" t="n">
         <v>25696</v>
@@ -2779,12 +2779,12 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>8.8%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>8.8%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="H18" t="n">
@@ -2811,7 +2811,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>291091</v>
+        <v>2910910000</v>
       </c>
       <c r="D19" t="n">
         <v>4980</v>
@@ -2821,12 +2821,12 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>1.7%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>1.7%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="H19" t="n">
@@ -2853,7 +2853,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>176745</v>
+        <v>1767450000</v>
       </c>
       <c r="D20" t="n">
         <v>14940</v>
@@ -2863,12 +2863,12 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>8.5%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>8.5%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="H20" t="n">
@@ -2895,7 +2895,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>155796</v>
+        <v>1557960000</v>
       </c>
       <c r="D21" t="n">
         <v>9960</v>
@@ -2905,12 +2905,12 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>6.4%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>6.4%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="H21" t="n">
@@ -2937,7 +2937,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>160474</v>
+        <v>1604740000</v>
       </c>
       <c r="D22" t="n">
         <v>14940</v>
@@ -2947,12 +2947,12 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>9.3%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>9.3%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="H22" t="n">
@@ -2979,7 +2979,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>265322</v>
+        <v>2653220000</v>
       </c>
       <c r="D23" t="n">
         <v>36178</v>
@@ -2989,12 +2989,12 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>13.6%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>13.6%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="H23" t="n">
@@ -3021,7 +3021,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>133802</v>
+        <v>1338020000</v>
       </c>
       <c r="D24" t="n">
         <v>33420</v>
@@ -3031,12 +3031,12 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>25.0%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>25.0%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="H24" t="n">
@@ -3063,7 +3063,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>128563</v>
+        <v>1285630000</v>
       </c>
       <c r="D25" t="n">
         <v>38000</v>
@@ -3073,12 +3073,12 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>29.6%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>29.6%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="H25" t="n">
@@ -3105,7 +3105,7 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>197614</v>
+        <v>1976140000</v>
       </c>
       <c r="D26" t="n">
         <v>24000</v>
@@ -3115,12 +3115,12 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>12.1%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>12.1%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="H26" t="n">
@@ -3147,7 +3147,7 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>192375</v>
+        <v>1923750000</v>
       </c>
       <c r="D27" t="n">
         <v>66400</v>
@@ -3157,12 +3157,12 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>34.5%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>34.5%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="H27" t="n">
@@ -3189,7 +3189,7 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>102098</v>
+        <v>1020980000</v>
       </c>
       <c r="D28" t="n">
         <v>0</v>
@@ -3231,7 +3231,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>102098</v>
+        <v>1020980000</v>
       </c>
       <c r="D29" t="n">
         <v>12000</v>
@@ -3241,12 +3241,12 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>11.8%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>11.8%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="H29" t="n">
@@ -3273,7 +3273,7 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>139041</v>
+        <v>1390410000</v>
       </c>
       <c r="D30" t="n">
         <v>6600</v>
@@ -3283,12 +3283,12 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>4.7%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>4.7%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="H30" t="n">
@@ -3315,7 +3315,7 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>102098</v>
+        <v>1020980000</v>
       </c>
       <c r="D31" t="n">
         <v>24088</v>
@@ -3325,12 +3325,12 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>23.6%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>23.6%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="H31" t="n">
@@ -3357,7 +3357,7 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>102098</v>
+        <v>1020980000</v>
       </c>
       <c r="D32" t="n">
         <v>43800</v>
@@ -3367,12 +3367,12 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>42.9%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>42.9%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="H32" t="n">
@@ -3399,7 +3399,7 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>102098</v>
+        <v>1020980000</v>
       </c>
       <c r="D33" t="n">
         <v>24800</v>
@@ -3409,12 +3409,12 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>24.3%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>24.3%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="H33" t="n">
@@ -3441,7 +3441,7 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>102098</v>
+        <v>1020980000</v>
       </c>
       <c r="D34" t="n">
         <v>0</v>
@@ -3483,7 +3483,7 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>102098</v>
+        <v>1020980000</v>
       </c>
       <c r="D35" t="n">
         <v>0</v>
@@ -3525,7 +3525,7 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>102103</v>
+        <v>1021030000</v>
       </c>
       <c r="D36" t="n">
         <v>0</v>
@@ -3664,7 +3664,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>60.7%</t>
+          <t>77.5%</t>
         </is>
       </c>
       <c r="F3" t="n">
@@ -3766,7 +3766,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>19.1%</t>
+          <t>20.3%</t>
         </is>
       </c>
       <c r="F6" t="n">
@@ -4378,7 +4378,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>23.5%</t>
+          <t>23.9%</t>
         </is>
       </c>
       <c r="F24" t="n">
@@ -4412,7 +4412,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>-4.1%</t>
+          <t>2.5%</t>
         </is>
       </c>
       <c r="F25" t="n">
@@ -4582,7 +4582,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>-5.2%</t>
+          <t>5.9%</t>
         </is>
       </c>
       <c r="F30" t="n">
@@ -4616,7 +4616,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>35.0%</t>
+          <t>43.2%</t>
         </is>
       </c>
       <c r="F31" t="n">
@@ -4684,7 +4684,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>7.4%</t>
+          <t>14.2%</t>
         </is>
       </c>
       <c r="F33" t="n">
@@ -4752,7 +4752,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>-3.2%</t>
+          <t>19.2%</t>
         </is>
       </c>
       <c r="F35" t="n">
@@ -4820,7 +4820,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>18.0%</t>
+          <t>20.0%</t>
         </is>
       </c>
       <c r="F37" t="n">
@@ -4990,7 +4990,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>-8.4%</t>
+          <t>1.7%</t>
         </is>
       </c>
       <c r="F42" t="n">
@@ -5160,7 +5160,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>40.5%</t>
+          <t>48.9%</t>
         </is>
       </c>
       <c r="F47" t="n">
@@ -5296,7 +5296,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>13.6%</t>
+          <t>20.9%</t>
         </is>
       </c>
       <c r="F51" t="n">
@@ -5704,7 +5704,7 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>23.4%</t>
+          <t>25.4%</t>
         </is>
       </c>
       <c r="F63" t="n">

</xml_diff>

<commit_message>
更新看板 10月11日 — KPI296.4万(16.0%) 净流水243.8万
</commit_message>
<xml_diff>
--- a/导出_总表.xlsx
+++ b/导出_总表.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q18"/>
+  <dimension ref="A1:Q19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1389,12 +1389,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>未映射</t>
+          <t>门店</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>未映射</t>
+          <t>望京</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -1404,29 +1404,33 @@
         <v>0</v>
       </c>
       <c r="E17" t="n">
-        <v>6500</v>
+        <v>0</v>
       </c>
       <c r="F17" t="n">
-        <v>-6500</v>
+        <v>0</v>
       </c>
       <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
       <c r="J17" t="n">
         <v>0</v>
       </c>
       <c r="K17" t="inlineStr"/>
       <c r="L17" t="n">
-        <v>-22514</v>
-      </c>
-      <c r="M17" t="inlineStr">
-        <is>
-          <t>-71.1%</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="M17" t="inlineStr"/>
       <c r="N17" t="inlineStr"/>
       <c r="O17" t="n">
-        <v>-6500</v>
+        <v>0</v>
       </c>
       <c r="P17" t="n">
         <v>0</v>
@@ -1438,65 +1442,114 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
+          <t>未映射</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>未映射</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" t="n">
+        <v>6500</v>
+      </c>
+      <c r="F18" t="n">
+        <v>-6500</v>
+      </c>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="n">
+        <v>0</v>
+      </c>
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" t="n">
+        <v>-22514</v>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>-71.1%</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr"/>
+      <c r="O18" t="n">
+        <v>-6500</v>
+      </c>
+      <c r="P18" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
           <t>合计</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B19" t="inlineStr">
         <is>
           <t>南区合计</t>
         </is>
       </c>
-      <c r="C18" t="n">
-        <v>17200000</v>
-      </c>
-      <c r="D18" t="n">
+      <c r="C19" t="n">
+        <v>18500000</v>
+      </c>
+      <c r="D19" t="n">
         <v>2964140</v>
       </c>
-      <c r="E18" t="n">
+      <c r="E19" t="n">
         <v>526074</v>
       </c>
-      <c r="F18" t="n">
+      <c r="F19" t="n">
         <v>2438066</v>
       </c>
-      <c r="G18" t="n">
-        <v>0</v>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>14.2%</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>14.2%</t>
-        </is>
-      </c>
-      <c r="J18" t="n">
+      <c r="G19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>16.0%</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>16.0%</t>
+        </is>
+      </c>
+      <c r="J19" t="n">
         <v>647841</v>
       </c>
-      <c r="K18" t="inlineStr">
+      <c r="K19" t="inlineStr">
         <is>
           <t>+357.5%</t>
         </is>
       </c>
-      <c r="L18" t="n">
+      <c r="L19" t="n">
         <v>-181067</v>
       </c>
-      <c r="M18" t="inlineStr">
+      <c r="M19" t="inlineStr">
         <is>
           <t>-1446.5%</t>
         </is>
       </c>
-      <c r="N18" t="n">
+      <c r="N19" t="n">
         <v>84957</v>
       </c>
-      <c r="O18" t="n">
+      <c r="O19" t="n">
         <v>747432</v>
       </c>
-      <c r="P18" t="n">
+      <c r="P19" t="n">
         <v>1605675</v>
       </c>
-      <c r="Q18" t="n">
+      <c r="Q19" t="n">
         <v>1192675</v>
       </c>
     </row>
@@ -1590,7 +1643,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1985,11 +2038,11 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>未映射</t>
+          <t>望京</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>-6500</v>
+        <v>0</v>
       </c>
       <c r="D19" t="n">
         <v>0</v>
@@ -2001,21 +2054,42 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
+          <t>分组</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>未映射</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>-6500</v>
+      </c>
+      <c r="D20" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
           <t>合计</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B21" t="inlineStr">
         <is>
           <t>南区合计</t>
         </is>
       </c>
-      <c r="C20" t="n">
+      <c r="C21" t="n">
         <v>747432</v>
       </c>
-      <c r="D20" t="n">
+      <c r="D21" t="n">
         <v>1605675</v>
       </c>
-      <c r="E20" t="n">
+      <c r="E21" t="n">
         <v>1192675</v>
       </c>
     </row>

</xml_diff>

<commit_message>
更新看板 10月12日 — KPI267.9万(17.9%) 净流水267.9万
Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/导出_总表.xlsx
+++ b/导出_总表.xlsx
@@ -541,12 +541,12 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>19.5%</t>
+          <t>16.0%</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>19.5%</t>
+          <t>16.0%</t>
         </is>
       </c>
       <c r="J2" t="n">
@@ -594,12 +594,12 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>7.8%</t>
+          <t>-1.3%</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>7.8%</t>
+          <t>-1.3%</t>
         </is>
       </c>
       <c r="J3" t="n">
@@ -647,12 +647,12 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>22.1%</t>
+          <t>18.8%</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>22.1%</t>
+          <t>18.8%</t>
         </is>
       </c>
       <c r="J4" t="n">
@@ -700,12 +700,12 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>22.4%</t>
+          <t>12.9%</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>22.4%</t>
+          <t>12.9%</t>
         </is>
       </c>
       <c r="J5" t="n">
@@ -737,7 +737,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>2500000</v>
+        <v>2000000</v>
       </c>
       <c r="D6" t="n">
         <v>596300</v>
@@ -751,12 +751,12 @@
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
-          <t>23.9%</t>
+          <t>28.0%</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>23.9%</t>
+          <t>28.0%</t>
         </is>
       </c>
       <c r="J6" t="n">
@@ -798,7 +798,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>500000</v>
+        <v>380000</v>
       </c>
       <c r="D7" t="n">
         <v>57135</v>
@@ -812,12 +812,12 @@
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
-          <t>11.4%</t>
+          <t>14.1%</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>11.4%</t>
+          <t>14.1%</t>
         </is>
       </c>
       <c r="J7" t="n">
@@ -859,7 +859,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>600000</v>
+        <v>400000</v>
       </c>
       <c r="D8" t="n">
         <v>257597</v>
@@ -873,12 +873,12 @@
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
-          <t>42.9%</t>
+          <t>64.1%</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>42.9%</t>
+          <t>64.1%</t>
         </is>
       </c>
       <c r="J8" t="n">
@@ -916,7 +916,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>1000000</v>
+        <v>800000</v>
       </c>
       <c r="D9" t="n">
         <v>205081</v>
@@ -930,12 +930,12 @@
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
-          <t>20.5%</t>
+          <t>21.5%</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>20.5%</t>
+          <t>21.5%</t>
         </is>
       </c>
       <c r="J9" t="n">
@@ -979,7 +979,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>1100000</v>
+        <v>1030000</v>
       </c>
       <c r="D10" t="n">
         <v>62025</v>
@@ -993,12 +993,12 @@
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
-          <t>5.6%</t>
+          <t>-1.3%</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>5.6%</t>
+          <t>-1.3%</t>
         </is>
       </c>
       <c r="J10" t="n">
@@ -1042,7 +1042,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>400000</v>
+        <v>260000</v>
       </c>
       <c r="D11" t="n">
         <v>18651</v>
@@ -1056,12 +1056,12 @@
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
         <is>
-          <t>4.7%</t>
+          <t>4.4%</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>4.7%</t>
+          <t>4.4%</t>
         </is>
       </c>
       <c r="J11" t="n">
@@ -1099,7 +1099,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>500000</v>
+        <v>400000</v>
       </c>
       <c r="D12" t="n">
         <v>220245</v>
@@ -1113,12 +1113,12 @@
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr">
         <is>
-          <t>44.0%</t>
+          <t>52.8%</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>44.0%</t>
+          <t>52.8%</t>
         </is>
       </c>
       <c r="J12" t="n">
@@ -1156,7 +1156,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1900000</v>
+        <v>1600000</v>
       </c>
       <c r="D13" t="n">
         <v>105001</v>
@@ -1170,12 +1170,12 @@
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr">
         <is>
-          <t>5.5%</t>
+          <t>5.9%</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>5.5%</t>
+          <t>5.9%</t>
         </is>
       </c>
       <c r="J13" t="n">
@@ -1219,7 +1219,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>1000000</v>
+        <v>900000</v>
       </c>
       <c r="D14" t="n">
         <v>529417</v>
@@ -1233,12 +1233,12 @@
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr">
         <is>
-          <t>52.9%</t>
+          <t>52.1%</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>52.9%</t>
+          <t>52.1%</t>
         </is>
       </c>
       <c r="J14" t="n">
@@ -1292,12 +1292,12 @@
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr">
         <is>
-          <t>19.4%</t>
+          <t>15.7%</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>19.4%</t>
+          <t>15.7%</t>
         </is>
       </c>
       <c r="J15" t="n">
@@ -1341,7 +1341,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>900000</v>
+        <v>700000</v>
       </c>
       <c r="D16" t="n">
         <v>48671</v>
@@ -1355,12 +1355,12 @@
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr">
         <is>
-          <t>5.4%</t>
+          <t>6.9%</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>5.4%</t>
+          <t>6.9%</t>
         </is>
       </c>
       <c r="J16" t="n">
@@ -1398,7 +1398,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>1300000</v>
+        <v>0</v>
       </c>
       <c r="D17" t="n">
         <v>0</v>
@@ -1500,7 +1500,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>18500000</v>
+        <v>15000000</v>
       </c>
       <c r="D19" t="n">
         <v>3338948</v>
@@ -1516,12 +1516,12 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>18.0%</t>
+          <t>17.9%</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>18.0%</t>
+          <t>17.9%</t>
         </is>
       </c>
       <c r="J19" t="n">
@@ -2171,22 +2171,22 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>3129120000</v>
+        <v>312912</v>
       </c>
       <c r="D2" t="n">
-        <v>84954</v>
+        <v>75177.3</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>24.0%</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>24.0%</t>
         </is>
       </c>
       <c r="H2" t="n">
@@ -2213,22 +2213,22 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>3026180000</v>
+        <v>302618</v>
       </c>
       <c r="D3" t="n">
-        <v>6260</v>
+        <v>1281</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>0.4%</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>0.4%</t>
         </is>
       </c>
       <c r="H3" t="n">
@@ -2255,22 +2255,22 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>2699380000</v>
+        <v>269938</v>
       </c>
       <c r="D4" t="n">
-        <v>34860</v>
+        <v>27357</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>10.1%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>10.1%</t>
         </is>
       </c>
       <c r="H4" t="n">
@@ -2297,22 +2297,22 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>1611540000</v>
+        <v>161154</v>
       </c>
       <c r="D5" t="n">
-        <v>22000</v>
+        <v>17319</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>10.7%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>10.7%</t>
         </is>
       </c>
       <c r="H5" t="n">
@@ -2339,22 +2339,22 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>1611540000</v>
+        <v>161154</v>
       </c>
       <c r="D6" t="n">
-        <v>21200</v>
+        <v>15520</v>
       </c>
       <c r="E6" t="n">
         <v>0</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>9.6%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>9.6%</t>
         </is>
       </c>
       <c r="H6" t="n">
@@ -2381,7 +2381,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>2424050000</v>
+        <v>242405</v>
       </c>
       <c r="D7" t="n">
         <v>4681</v>
@@ -2391,12 +2391,12 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>1.9%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>1.9%</t>
         </is>
       </c>
       <c r="H7" t="n">
@@ -2423,22 +2423,22 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>1891360000</v>
+        <v>189136</v>
       </c>
       <c r="D8" t="n">
-        <v>4980</v>
+        <v>1000</v>
       </c>
       <c r="E8" t="n">
         <v>0</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>0.5%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>0.5%</t>
         </is>
       </c>
       <c r="H8" t="n">
@@ -2465,22 +2465,22 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>3336160000</v>
+        <v>333616</v>
       </c>
       <c r="D9" t="n">
-        <v>42936</v>
+        <v>-10960.67</v>
       </c>
       <c r="E9" t="n">
         <v>0</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>-3.3%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>-3.3%</t>
         </is>
       </c>
       <c r="H9" t="n">
@@ -2507,7 +2507,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>2714400000</v>
+        <v>271440</v>
       </c>
       <c r="D10" t="n">
         <v>0</v>
@@ -2549,22 +2549,22 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>2714400000</v>
+        <v>271440</v>
       </c>
       <c r="D11" t="n">
-        <v>10160</v>
+        <v>160</v>
       </c>
       <c r="E11" t="n">
         <v>0</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>0.1%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>0.1%</t>
         </is>
       </c>
       <c r="H11" t="n">
@@ -2591,7 +2591,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>2392460000</v>
+        <v>239246</v>
       </c>
       <c r="D12" t="n">
         <v>14940</v>
@@ -2601,12 +2601,12 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>6.2%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>6.2%</t>
         </is>
       </c>
       <c r="H12" t="n">
@@ -2633,7 +2633,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>2277770000</v>
+        <v>227777</v>
       </c>
       <c r="D13" t="n">
         <v>0</v>
@@ -2675,22 +2675,22 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>2070510000</v>
+        <v>207051</v>
       </c>
       <c r="D14" t="n">
-        <v>14940</v>
+        <v>-40823</v>
       </c>
       <c r="E14" t="n">
         <v>0</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>-19.7%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>-19.7%</t>
         </is>
       </c>
       <c r="H14" t="n">
@@ -2717,7 +2717,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>1472910000</v>
+        <v>147291</v>
       </c>
       <c r="D15" t="n">
         <v>6600</v>
@@ -2727,12 +2727,12 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>4.5%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>4.5%</t>
         </is>
       </c>
       <c r="H15" t="n">
@@ -2759,7 +2759,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>2790500000</v>
+        <v>279050</v>
       </c>
       <c r="D16" t="n">
         <v>34900</v>
@@ -2769,12 +2769,12 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>12.5%</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>12.5%</t>
         </is>
       </c>
       <c r="H16" t="n">
@@ -2801,22 +2801,22 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>2855170000</v>
+        <v>285517</v>
       </c>
       <c r="D17" t="n">
-        <v>89054</v>
+        <v>84489</v>
       </c>
       <c r="E17" t="n">
         <v>0</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>29.6%</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>29.6%</t>
         </is>
       </c>
       <c r="H17" t="n">
@@ -2843,7 +2843,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>2906430000</v>
+        <v>290643</v>
       </c>
       <c r="D18" t="n">
         <v>25696</v>
@@ -2853,12 +2853,12 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>8.8%</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>8.8%</t>
         </is>
       </c>
       <c r="H18" t="n">
@@ -2885,22 +2885,22 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>2910910000</v>
+        <v>291091</v>
       </c>
       <c r="D19" t="n">
-        <v>4980</v>
+        <v>-10000</v>
       </c>
       <c r="E19" t="n">
         <v>0</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>-3.4%</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>-3.4%</t>
         </is>
       </c>
       <c r="H19" t="n">
@@ -2927,22 +2927,22 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>1767450000</v>
+        <v>176745</v>
       </c>
       <c r="D20" t="n">
-        <v>19920</v>
+        <v>15493.33</v>
       </c>
       <c r="E20" t="n">
         <v>0</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>8.8%</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>8.8%</t>
         </is>
       </c>
       <c r="H20" t="n">
@@ -2969,22 +2969,22 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>1557960000</v>
+        <v>155796</v>
       </c>
       <c r="D21" t="n">
-        <v>14940</v>
+        <v>9960</v>
       </c>
       <c r="E21" t="n">
         <v>0</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>6.4%</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>6.4%</t>
         </is>
       </c>
       <c r="H21" t="n">
@@ -3011,22 +3011,22 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>1604740000</v>
+        <v>160474</v>
       </c>
       <c r="D22" t="n">
-        <v>19920</v>
+        <v>9940</v>
       </c>
       <c r="E22" t="n">
         <v>0</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>6.2%</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>6.2%</t>
         </is>
       </c>
       <c r="H22" t="n">
@@ -3053,22 +3053,22 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>2653220000</v>
+        <v>265322</v>
       </c>
       <c r="D23" t="n">
-        <v>36178</v>
+        <v>26218</v>
       </c>
       <c r="E23" t="n">
         <v>0</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>9.9%</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>9.9%</t>
         </is>
       </c>
       <c r="H23" t="n">
@@ -3095,22 +3095,22 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>1338020000</v>
+        <v>133802</v>
       </c>
       <c r="D24" t="n">
-        <v>33420</v>
+        <v>6600</v>
       </c>
       <c r="E24" t="n">
         <v>0</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>4.9%</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>4.9%</t>
         </is>
       </c>
       <c r="H24" t="n">
@@ -3137,22 +3137,22 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>1285630000</v>
+        <v>128563</v>
       </c>
       <c r="D25" t="n">
-        <v>44600</v>
+        <v>25800</v>
       </c>
       <c r="E25" t="n">
         <v>0</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>20.1%</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>20.1%</t>
         </is>
       </c>
       <c r="H25" t="n">
@@ -3179,7 +3179,7 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>1976140000</v>
+        <v>197614</v>
       </c>
       <c r="D26" t="n">
         <v>24000</v>
@@ -3189,12 +3189,12 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>12.1%</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>12.1%</t>
         </is>
       </c>
       <c r="H26" t="n">
@@ -3221,22 +3221,22 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>1923750000</v>
+        <v>192375</v>
       </c>
       <c r="D27" t="n">
-        <v>66400</v>
+        <v>57400</v>
       </c>
       <c r="E27" t="n">
         <v>0</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>29.8%</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>29.8%</t>
         </is>
       </c>
       <c r="H27" t="n">
@@ -3263,7 +3263,7 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>1020980000</v>
+        <v>102098</v>
       </c>
       <c r="D28" t="n">
         <v>6600</v>
@@ -3273,12 +3273,12 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>6.5%</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>6.5%</t>
         </is>
       </c>
       <c r="H28" t="n">
@@ -3305,7 +3305,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>1020980000</v>
+        <v>102098</v>
       </c>
       <c r="D29" t="n">
         <v>12000</v>
@@ -3315,12 +3315,12 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>11.8%</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>11.8%</t>
         </is>
       </c>
       <c r="H29" t="n">
@@ -3347,7 +3347,7 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>1390410000</v>
+        <v>139041</v>
       </c>
       <c r="D30" t="n">
         <v>25200</v>
@@ -3357,12 +3357,12 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>18.1%</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>18.1%</t>
         </is>
       </c>
       <c r="H30" t="n">
@@ -3389,22 +3389,22 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>1020980000</v>
+        <v>102098</v>
       </c>
       <c r="D31" t="n">
-        <v>24088</v>
+        <v>20088</v>
       </c>
       <c r="E31" t="n">
         <v>0</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>19.7%</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>19.7%</t>
         </is>
       </c>
       <c r="H31" t="n">
@@ -3431,7 +3431,7 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>1020980000</v>
+        <v>102098</v>
       </c>
       <c r="D32" t="n">
         <v>43800</v>
@@ -3441,12 +3441,12 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>42.9%</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>42.9%</t>
         </is>
       </c>
       <c r="H32" t="n">
@@ -3473,7 +3473,7 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>1020980000</v>
+        <v>102098</v>
       </c>
       <c r="D33" t="n">
         <v>34800</v>
@@ -3483,12 +3483,12 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>34.1%</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>34.1%</t>
         </is>
       </c>
       <c r="H33" t="n">
@@ -3515,7 +3515,7 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>1020980000</v>
+        <v>102098</v>
       </c>
       <c r="D34" t="n">
         <v>0</v>
@@ -3557,7 +3557,7 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>1020980000</v>
+        <v>102098</v>
       </c>
       <c r="D35" t="n">
         <v>0</v>
@@ -3599,7 +3599,7 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>1021030000</v>
+        <v>102103</v>
       </c>
       <c r="D36" t="n">
         <v>0</v>
@@ -3734,11 +3734,11 @@
         <v>350000</v>
       </c>
       <c r="D3" t="n">
-        <v>281908</v>
+        <v>223108</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>80.5%</t>
+          <t>63.7%</t>
         </is>
       </c>
       <c r="F3" t="n">
@@ -3836,11 +3836,11 @@
         <v>140000</v>
       </c>
       <c r="D6" t="n">
-        <v>28392</v>
+        <v>26792</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>20.3%</t>
+          <t>19.1%</t>
         </is>
       </c>
       <c r="F6" t="n">
@@ -3938,11 +3938,11 @@
         <v>140000</v>
       </c>
       <c r="D9" t="n">
-        <v>0</v>
+        <v>-598</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>-0.4%</t>
         </is>
       </c>
       <c r="F9" t="n">
@@ -4448,11 +4448,11 @@
         <v>190000</v>
       </c>
       <c r="D24" t="n">
-        <v>55419.88</v>
+        <v>54623.88</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>29.2%</t>
+          <t>28.7%</t>
         </is>
       </c>
       <c r="F24" t="n">
@@ -4482,11 +4482,11 @@
         <v>150000</v>
       </c>
       <c r="D25" t="n">
-        <v>3790</v>
+        <v>-6210</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2.5%</t>
+          <t>-4.1%</t>
         </is>
       </c>
       <c r="F25" t="n">
@@ -4652,11 +4652,11 @@
         <v>130000</v>
       </c>
       <c r="D30" t="n">
-        <v>7700</v>
+        <v>-6800</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>5.9%</t>
+          <t>-5.2%</t>
         </is>
       </c>
       <c r="F30" t="n">
@@ -4686,11 +4686,11 @@
         <v>115000</v>
       </c>
       <c r="D31" t="n">
-        <v>49696</v>
+        <v>40196</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>43.2%</t>
+          <t>35.0%</t>
         </is>
       </c>
       <c r="F31" t="n">
@@ -4754,11 +4754,11 @@
         <v>125000</v>
       </c>
       <c r="D33" t="n">
-        <v>17796</v>
+        <v>9296</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>14.2%</t>
+          <t>7.4%</t>
         </is>
       </c>
       <c r="F33" t="n">
@@ -4822,11 +4822,11 @@
         <v>150000</v>
       </c>
       <c r="D35" t="n">
-        <v>39660</v>
+        <v>6060</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>26.4%</t>
+          <t>4.0%</t>
         </is>
       </c>
       <c r="F35" t="n">
@@ -4890,11 +4890,11 @@
         <v>100000</v>
       </c>
       <c r="D37" t="n">
-        <v>20000</v>
+        <v>16040</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>20.0%</t>
+          <t>16.0%</t>
         </is>
       </c>
       <c r="F37" t="n">
@@ -5060,11 +5060,11 @@
         <v>70000</v>
       </c>
       <c r="D42" t="n">
-        <v>1200</v>
+        <v>-5883.33</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>1.7%</t>
+          <t>-8.4%</t>
         </is>
       </c>
       <c r="F42" t="n">
@@ -5230,11 +5230,11 @@
         <v>110000</v>
       </c>
       <c r="D47" t="n">
-        <v>118590</v>
+        <v>109390</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>107.8%</t>
+          <t>99.4%</t>
         </is>
       </c>
       <c r="F47" t="n">
@@ -5366,11 +5366,11 @@
         <v>160000</v>
       </c>
       <c r="D51" t="n">
-        <v>33564.8</v>
+        <v>21964.8</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>21.0%</t>
+          <t>13.7%</t>
         </is>
       </c>
       <c r="F51" t="n">
@@ -5638,11 +5638,11 @@
         <v>70000</v>
       </c>
       <c r="D59" t="n">
-        <v>65998</v>
+        <v>64998</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>94.3%</t>
+          <t>92.9%</t>
         </is>
       </c>
       <c r="F59" t="n">
@@ -5774,11 +5774,11 @@
         <v>170000</v>
       </c>
       <c r="D63" t="n">
-        <v>43190</v>
+        <v>39790</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>25.4%</t>
+          <t>23.4%</t>
         </is>
       </c>
       <c r="F63" t="n">

</xml_diff>

<commit_message>
更新看板 10月12日 — KPI267.9万(17.5%) 净流水267.9万
Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/导出_总表.xlsx
+++ b/导出_总表.xlsx
@@ -1500,7 +1500,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>15000000</v>
+        <v>15270000</v>
       </c>
       <c r="D19" t="n">
         <v>3338948</v>
@@ -1516,12 +1516,12 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>17.9%</t>
+          <t>17.5%</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>17.9%</t>
+          <t>17.5%</t>
         </is>
       </c>
       <c r="J19" t="n">

</xml_diff>

<commit_message>
更新看板 10月12日 — KPI267.9万(14.5%) 净流水267.9万
Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/导出_总表.xlsx
+++ b/导出_总表.xlsx
@@ -737,7 +737,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>2000000</v>
+        <v>2500000</v>
       </c>
       <c r="D6" t="n">
         <v>596300</v>
@@ -751,12 +751,12 @@
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
-          <t>28.0%</t>
+          <t>22.4%</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>28.0%</t>
+          <t>22.4%</t>
         </is>
       </c>
       <c r="J6" t="n">
@@ -798,7 +798,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>380000</v>
+        <v>500000</v>
       </c>
       <c r="D7" t="n">
         <v>57135</v>
@@ -812,12 +812,12 @@
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
-          <t>14.1%</t>
+          <t>10.7%</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>14.1%</t>
+          <t>10.7%</t>
         </is>
       </c>
       <c r="J7" t="n">
@@ -859,7 +859,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>400000</v>
+        <v>600000</v>
       </c>
       <c r="D8" t="n">
         <v>257597</v>
@@ -873,12 +873,12 @@
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
-          <t>64.1%</t>
+          <t>42.8%</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>64.1%</t>
+          <t>42.8%</t>
         </is>
       </c>
       <c r="J8" t="n">
@@ -916,7 +916,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>800000</v>
+        <v>1000000</v>
       </c>
       <c r="D9" t="n">
         <v>205081</v>
@@ -930,12 +930,12 @@
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
-          <t>21.5%</t>
+          <t>17.2%</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>21.5%</t>
+          <t>17.2%</t>
         </is>
       </c>
       <c r="J9" t="n">
@@ -979,7 +979,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>1030000</v>
+        <v>1100000</v>
       </c>
       <c r="D10" t="n">
         <v>62025</v>
@@ -1042,7 +1042,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>260000</v>
+        <v>400000</v>
       </c>
       <c r="D11" t="n">
         <v>18651</v>
@@ -1056,12 +1056,12 @@
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
         <is>
-          <t>4.4%</t>
+          <t>2.9%</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>4.4%</t>
+          <t>2.9%</t>
         </is>
       </c>
       <c r="J11" t="n">
@@ -1099,7 +1099,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>400000</v>
+        <v>500000</v>
       </c>
       <c r="D12" t="n">
         <v>220245</v>
@@ -1113,12 +1113,12 @@
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr">
         <is>
-          <t>52.8%</t>
+          <t>42.2%</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>52.8%</t>
+          <t>42.2%</t>
         </is>
       </c>
       <c r="J12" t="n">
@@ -1156,7 +1156,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1600000</v>
+        <v>1900000</v>
       </c>
       <c r="D13" t="n">
         <v>105001</v>
@@ -1170,12 +1170,12 @@
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr">
         <is>
-          <t>5.9%</t>
+          <t>5.0%</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>5.9%</t>
+          <t>5.0%</t>
         </is>
       </c>
       <c r="J13" t="n">
@@ -1219,7 +1219,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>900000</v>
+        <v>1000000</v>
       </c>
       <c r="D14" t="n">
         <v>529417</v>
@@ -1233,12 +1233,12 @@
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr">
         <is>
-          <t>52.1%</t>
+          <t>46.9%</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>52.1%</t>
+          <t>46.9%</t>
         </is>
       </c>
       <c r="J14" t="n">
@@ -1341,7 +1341,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>700000</v>
+        <v>900000</v>
       </c>
       <c r="D16" t="n">
         <v>48671</v>
@@ -1355,12 +1355,12 @@
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr">
         <is>
-          <t>6.9%</t>
+          <t>5.3%</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>6.9%</t>
+          <t>5.3%</t>
         </is>
       </c>
       <c r="J16" t="n">
@@ -1398,7 +1398,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>0</v>
+        <v>1300000</v>
       </c>
       <c r="D17" t="n">
         <v>0</v>
@@ -1500,7 +1500,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>15270000</v>
+        <v>18500000</v>
       </c>
       <c r="D19" t="n">
         <v>3338948</v>
@@ -1516,12 +1516,12 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>17.5%</t>
+          <t>14.5%</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>17.5%</t>
+          <t>14.5%</t>
         </is>
       </c>
       <c r="J19" t="n">

</xml_diff>

<commit_message>
更新看板 10月12日 — KPI267.9万(15.6%) 净流水267.9万
Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/导出_总表.xlsx
+++ b/导出_总表.xlsx
@@ -1500,7 +1500,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>18500000</v>
+        <v>17200000</v>
       </c>
       <c r="D19" t="n">
         <v>3338948</v>
@@ -1516,12 +1516,12 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>14.5%</t>
+          <t>15.6%</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>14.5%</t>
+          <t>15.6%</t>
         </is>
       </c>
       <c r="J19" t="n">

</xml_diff>

<commit_message>
更新看板 10月22日 — KPI1027.7万(55.6%) 净流水838.1万
Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/导出_总表.xlsx
+++ b/导出_总表.xlsx
@@ -4121,7 +4121,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4132,22 +4132,27 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>呼出</t>
+          <t>通话数/日</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>90s以上</t>
+          <t>≥90S通话数</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>时长(分)</t>
+          <t>≥20分钟通话数</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>加微信</t>
+          <t>云客通话数</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>企业微信通话数</t>
         </is>
       </c>
     </row>
@@ -4158,16 +4163,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>216</v>
+        <v>306</v>
       </c>
       <c r="C2" t="n">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="D2" t="n">
-        <v>567.2</v>
+        <v>17</v>
       </c>
       <c r="E2" t="n">
-        <v>2835</v>
+        <v>269</v>
+      </c>
+      <c r="F2" t="n">
+        <v>37</v>
       </c>
     </row>
     <row r="3">
@@ -4177,16 +4185,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>20</v>
+        <v>43</v>
       </c>
       <c r="C3" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="D3" t="n">
-        <v>340.6</v>
+        <v>7</v>
       </c>
       <c r="E3" t="n">
-        <v>95</v>
+        <v>37</v>
+      </c>
+      <c r="F3" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="4">
@@ -4196,16 +4207,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>660</v>
+        <v>446</v>
       </c>
       <c r="C4" t="n">
-        <v>111</v>
+        <v>91</v>
       </c>
       <c r="D4" t="n">
-        <v>1388.4</v>
+        <v>11</v>
       </c>
       <c r="E4" t="n">
-        <v>3311</v>
+        <v>406</v>
+      </c>
+      <c r="F4" t="n">
+        <v>40</v>
       </c>
     </row>
     <row r="5">
@@ -4215,16 +4229,19 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0</v>
+        <v>132</v>
       </c>
       <c r="C5" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="D5" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E5" t="n">
-        <v>0</v>
+        <v>131</v>
+      </c>
+      <c r="F5" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -6972,7 +6989,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>芊雅</t>
+          <t>王芊雅</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -8264,30 +8281,30 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>黄惠作</t>
+          <t>黄慧作</t>
         </is>
       </c>
       <c r="C49" t="n">
         <v>200000</v>
       </c>
       <c r="D49" t="n">
-        <v>0</v>
+        <v>197010</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>98.5%</t>
         </is>
       </c>
       <c r="F49" t="n">
-        <v>0</v>
+        <v>54910</v>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>27.9%</t>
         </is>
       </c>
       <c r="H49" t="n">
-        <v>0</v>
+        <v>142100</v>
       </c>
     </row>
     <row r="50">

</xml_diff>

<commit_message>
更新看板 10月30日 — KPI1557.5万(84.2%) 净流水1277.8万
Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/导出_总表.xlsx
+++ b/导出_总表.xlsx
@@ -725,19 +725,19 @@
         </is>
       </c>
       <c r="J5" t="n">
-        <v>1133732</v>
+        <v>1491270</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>+67.0%</t>
+          <t>+27.0%</t>
         </is>
       </c>
       <c r="L5" t="n">
-        <v>613316</v>
+        <v>959874</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>+135.4%</t>
+          <t>+50.4%</t>
         </is>
       </c>
       <c r="N5" t="inlineStr"/>
@@ -1571,19 +1571,19 @@
         </is>
       </c>
       <c r="J19" t="n">
-        <v>10846084</v>
+        <v>11203622</v>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>+43.6%</t>
+          <t>+39.0%</t>
         </is>
       </c>
       <c r="L19" t="n">
-        <v>9109939</v>
+        <v>9456497</v>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>+40.3%</t>
+          <t>+35.1%</t>
         </is>
       </c>
       <c r="N19" t="n">
@@ -4932,7 +4932,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J44"/>
+  <dimension ref="A1:J45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6460,43 +6460,43 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>观澜组</t>
+          <t>观鼎组</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>姚闯</t>
+          <t>江敏</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>200000</v>
+        <v>0</v>
       </c>
       <c r="D37" t="n">
-        <v>102694</v>
+        <v>215700</v>
       </c>
       <c r="E37" t="n">
         <v>0</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>51.3%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>51.3%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="H37" t="n">
-        <v>33460</v>
+        <v>16400</v>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>32.6%</t>
+          <t>7.6%</t>
         </is>
       </c>
       <c r="J37" t="n">
-        <v>69234</v>
+        <v>199300</v>
       </c>
     </row>
     <row r="38">
@@ -6507,38 +6507,38 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>魏恺志</t>
+          <t>姚闯</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>100000</v>
+        <v>200000</v>
       </c>
       <c r="D38" t="n">
-        <v>8280</v>
+        <v>102694</v>
       </c>
       <c r="E38" t="n">
         <v>0</v>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>8.3%</t>
+          <t>51.3%</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>8.3%</t>
+          <t>51.3%</t>
         </is>
       </c>
       <c r="H38" t="n">
-        <v>2160</v>
+        <v>33460</v>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>26.1%</t>
+          <t>32.6%</t>
         </is>
       </c>
       <c r="J38" t="n">
-        <v>6120</v>
+        <v>69234</v>
       </c>
     </row>
     <row r="39">
@@ -6549,38 +6549,38 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>杨旺忠</t>
+          <t>魏恺志</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>250000</v>
+        <v>100000</v>
       </c>
       <c r="D39" t="n">
-        <v>93640</v>
+        <v>8280</v>
       </c>
       <c r="E39" t="n">
         <v>0</v>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>37.5%</t>
+          <t>8.3%</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>37.5%</t>
+          <t>8.3%</t>
         </is>
       </c>
       <c r="H39" t="n">
-        <v>4060</v>
+        <v>2160</v>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>4.3%</t>
+          <t>26.1%</t>
         </is>
       </c>
       <c r="J39" t="n">
-        <v>89580</v>
+        <v>6120</v>
       </c>
     </row>
     <row r="40">
@@ -6591,38 +6591,38 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>闫浩</t>
+          <t>杨旺忠</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>0</v>
+        <v>250000</v>
       </c>
       <c r="D40" t="n">
-        <v>0</v>
+        <v>93640</v>
       </c>
       <c r="E40" t="n">
         <v>0</v>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>37.5%</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>37.5%</t>
         </is>
       </c>
       <c r="H40" t="n">
-        <v>0</v>
+        <v>4060</v>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>4.3%</t>
         </is>
       </c>
       <c r="J40" t="n">
-        <v>0</v>
+        <v>89580</v>
       </c>
     </row>
     <row r="41">
@@ -6633,38 +6633,38 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>余文静</t>
+          <t>闫浩</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>250000</v>
+        <v>0</v>
       </c>
       <c r="D41" t="n">
-        <v>126380</v>
+        <v>0</v>
       </c>
       <c r="E41" t="n">
         <v>0</v>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>50.6%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>50.6%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="H41" t="n">
-        <v>4240</v>
+        <v>0</v>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>3.4%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="J41" t="n">
-        <v>122140</v>
+        <v>0</v>
       </c>
     </row>
     <row r="42">
@@ -6675,38 +6675,38 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>陈鑫</t>
+          <t>余文静</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>400000</v>
+        <v>250000</v>
       </c>
       <c r="D42" t="n">
-        <v>436890</v>
+        <v>126380</v>
       </c>
       <c r="E42" t="n">
         <v>0</v>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>109.2%</t>
+          <t>50.6%</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>109.2%</t>
+          <t>50.6%</t>
         </is>
       </c>
       <c r="H42" t="n">
-        <v>1980</v>
+        <v>4240</v>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>0.5%</t>
+          <t>3.4%</t>
         </is>
       </c>
       <c r="J42" t="n">
-        <v>434910</v>
+        <v>122140</v>
       </c>
     </row>
     <row r="43">
@@ -6717,38 +6717,38 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>吴云龙</t>
+          <t>陈鑫</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>200000</v>
+        <v>400000</v>
       </c>
       <c r="D43" t="n">
-        <v>57280</v>
+        <v>436890</v>
       </c>
       <c r="E43" t="n">
         <v>0</v>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>28.6%</t>
+          <t>109.2%</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>28.6%</t>
+          <t>109.2%</t>
         </is>
       </c>
       <c r="H43" t="n">
-        <v>0</v>
+        <v>1980</v>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>0.5%</t>
         </is>
       </c>
       <c r="J43" t="n">
-        <v>57280</v>
+        <v>434910</v>
       </c>
     </row>
     <row r="44">
@@ -6759,37 +6759,79 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>龙刚</t>
+          <t>吴云龙</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>100000</v>
+        <v>200000</v>
       </c>
       <c r="D44" t="n">
-        <v>2190</v>
+        <v>57280</v>
       </c>
       <c r="E44" t="n">
         <v>0</v>
       </c>
       <c r="F44" t="inlineStr">
         <is>
+          <t>28.6%</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>28.6%</t>
+        </is>
+      </c>
+      <c r="H44" t="n">
+        <v>0</v>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="J44" t="n">
+        <v>57280</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>观澜组</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>龙刚</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>100000</v>
+      </c>
+      <c r="D45" t="n">
+        <v>2190</v>
+      </c>
+      <c r="E45" t="n">
+        <v>0</v>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
           <t>2.2%</t>
         </is>
       </c>
-      <c r="G44" t="inlineStr">
+      <c r="G45" t="inlineStr">
         <is>
           <t>2.2%</t>
         </is>
       </c>
-      <c r="H44" t="n">
+      <c r="H45" t="n">
         <v>2980</v>
       </c>
-      <c r="I44" t="inlineStr">
+      <c r="I45" t="inlineStr">
         <is>
           <t>136.1%</t>
         </is>
       </c>
-      <c r="J44" t="n">
+      <c r="J45" t="n">
         <v>-790</v>
       </c>
     </row>

</xml_diff>